<commit_message>
feat: Optimasi penjadwalan Web Worker, perbaikan bug type casting, & penambahan filter Mapel pada Rekapitulasi
</commit_message>
<xml_diff>
--- a/public/template_data_siswa.xlsx
+++ b/public/template_data_siswa.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DiTa\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\app-firebase\sekolahPintar\smart-school-backend\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2563632F-5AA0-4586-BDDF-592A83CA1579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5112D972-7075-495F-9846-CF3A92C51B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
   <si>
     <t>Kode Siswa</t>
   </si>
@@ -100,6 +100,9 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>Alamat</t>
   </si>
 </sst>
 </file>
@@ -505,8 +508,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.625" customWidth="1"/>
     <col min="2" max="2" width="10.125" customWidth="1"/>
@@ -517,9 +520,10 @@
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="13.75" customWidth="1"/>
     <col min="9" max="9" width="13.5" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -547,8 +551,11 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>

</xml_diff>